<commit_message>
chore(dados): atualiza planilhas de importação de convênios
</commit_message>
<xml_diff>
--- a/docs/sespa.xlsx
+++ b/docs/sespa.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c83854e6706cf50b/Documentos/Seplad/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c83854e6706cf50b/Seplad/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="96" documentId="8_{063CAB35-503D-47C0-82A2-0769B90FB030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4355B56-C920-4B30-87CE-6353CC602440}"/>
+  <xr:revisionPtr revIDLastSave="130" documentId="8_{063CAB35-503D-47C0-82A2-0769B90FB030}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6D7E229D-1C60-41B5-94FB-A52AC09B5DC3}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8658C97B-32F7-49BC-91D6-938C503E2FBD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{8658C97B-32F7-49BC-91D6-938C503E2FBD}"/>
   </bookViews>
   <sheets>
     <sheet name="lista" sheetId="1" r:id="rId1"/>
@@ -73,9 +73,6 @@
     <t>MOJU</t>
   </si>
   <si>
-    <t xml:space="preserve">ALMEIRIM </t>
-  </si>
-  <si>
     <t xml:space="preserve">BREVES </t>
   </si>
   <si>
@@ -579,6 +576,9 @@
   </si>
   <si>
     <t>CONSTRUÇÃO DO HOSPITAL MUNICIPAL DE URUARÁ</t>
+  </si>
+  <si>
+    <t>ALMEIRIM</t>
   </si>
 </sst>
 </file>
@@ -1064,22 +1064,22 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H1" t="s">
         <v>42</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>43</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -1087,20 +1087,20 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E2" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G2" t="s">
         <v>8</v>
@@ -1126,20 +1126,20 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>179</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>179</v>
       </c>
       <c r="D3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E3" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G3" t="s">
         <v>8</v>
@@ -1165,20 +1165,20 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E4" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2024</v>
       </c>
       <c r="F4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G4" t="s">
         <v>8</v>
@@ -1204,23 +1204,23 @@
         <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E5" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2023</v>
       </c>
       <c r="F5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H5" s="1">
         <v>45159</v>
@@ -1243,20 +1243,20 @@
         <v>6</v>
       </c>
       <c r="B6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E6" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2023</v>
       </c>
       <c r="F6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G6" t="s">
         <v>8</v>
@@ -1282,20 +1282,20 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E7" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2023</v>
       </c>
       <c r="F7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G7" t="s">
         <v>8</v>
@@ -1321,23 +1321,23 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E8" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2024</v>
       </c>
       <c r="F8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H8" s="1">
         <v>45478</v>
@@ -1360,20 +1360,20 @@
         <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E9" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G9" t="s">
         <v>8</v>
@@ -1399,20 +1399,20 @@
         <v>6</v>
       </c>
       <c r="B10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E10" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G10" t="s">
         <v>8</v>
@@ -1438,20 +1438,20 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E11" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2025</v>
       </c>
       <c r="F11" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G11" t="s">
         <v>8</v>
@@ -1477,20 +1477,20 @@
         <v>6</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D12" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E12" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G12" t="s">
         <v>8</v>
@@ -1516,20 +1516,20 @@
         <v>6</v>
       </c>
       <c r="B13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D13" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E13" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F13" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G13" t="s">
         <v>8</v>
@@ -1561,14 +1561,14 @@
         <v>7</v>
       </c>
       <c r="D14" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E14" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2021</v>
       </c>
       <c r="F14" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G14" t="s">
         <v>8</v>
@@ -1594,20 +1594,20 @@
         <v>6</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E15" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F15" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G15" t="s">
         <v>8</v>
@@ -1633,20 +1633,20 @@
         <v>6</v>
       </c>
       <c r="B16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D16" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E16" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2024</v>
       </c>
       <c r="F16" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G16" t="s">
         <v>8</v>
@@ -1672,20 +1672,20 @@
         <v>6</v>
       </c>
       <c r="B17" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C17" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D17" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E17" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2024</v>
       </c>
       <c r="F17" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G17" t="s">
         <v>8</v>
@@ -1711,20 +1711,20 @@
         <v>6</v>
       </c>
       <c r="B18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D18" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E18" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F18" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G18" t="s">
         <v>8</v>
@@ -1756,14 +1756,14 @@
         <v>10</v>
       </c>
       <c r="D19" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E19" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F19" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G19" t="s">
         <v>8</v>
@@ -1789,20 +1789,20 @@
         <v>6</v>
       </c>
       <c r="B20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D20" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E20" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2025</v>
       </c>
       <c r="F20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="G20" t="s">
         <v>8</v>
@@ -1828,20 +1828,20 @@
         <v>6</v>
       </c>
       <c r="B21" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C21" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D21" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E21" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F21" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G21" t="s">
         <v>8</v>
@@ -1867,20 +1867,20 @@
         <v>6</v>
       </c>
       <c r="B22" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C22" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D22" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E22" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F22" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G22" t="s">
         <v>8</v>
@@ -1906,20 +1906,20 @@
         <v>6</v>
       </c>
       <c r="B23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D23" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E23" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F23" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G23" t="s">
         <v>8</v>
@@ -1945,20 +1945,20 @@
         <v>6</v>
       </c>
       <c r="B24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D24" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="E24" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F24" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G24" t="s">
         <v>8</v>
@@ -1984,20 +1984,20 @@
         <v>6</v>
       </c>
       <c r="B25" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C25" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D25" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E25" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F25" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G25" t="s">
         <v>8</v>
@@ -2023,20 +2023,20 @@
         <v>6</v>
       </c>
       <c r="B26" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C26" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D26" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E26" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F26" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G26" t="s">
         <v>8</v>
@@ -2062,20 +2062,20 @@
         <v>6</v>
       </c>
       <c r="B27" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C27" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D27" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E27" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F27" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G27" t="s">
         <v>8</v>
@@ -2101,20 +2101,20 @@
         <v>6</v>
       </c>
       <c r="B28" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C28" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D28" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E28" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2024</v>
       </c>
       <c r="F28" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G28" t="s">
         <v>8</v>
@@ -2146,14 +2146,14 @@
         <v>9</v>
       </c>
       <c r="D29" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E29" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F29" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G29" t="s">
         <v>8</v>
@@ -2179,20 +2179,20 @@
         <v>6</v>
       </c>
       <c r="B30" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C30" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D30" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E30" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F30" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G30" t="s">
         <v>8</v>
@@ -2218,20 +2218,20 @@
         <v>6</v>
       </c>
       <c r="B31" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C31" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D31" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E31" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2023</v>
       </c>
       <c r="F31" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G31" t="s">
         <v>8</v>
@@ -2257,20 +2257,20 @@
         <v>6</v>
       </c>
       <c r="B32" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C32" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D32" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E32" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F32" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="G32" t="s">
         <v>8</v>
@@ -2296,20 +2296,20 @@
         <v>6</v>
       </c>
       <c r="B33" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C33" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D33" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E33" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F33" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G33" t="s">
         <v>8</v>
@@ -2335,20 +2335,20 @@
         <v>6</v>
       </c>
       <c r="B34" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C34" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D34" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E34" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F34" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G34" t="s">
         <v>8</v>
@@ -2374,20 +2374,20 @@
         <v>6</v>
       </c>
       <c r="B35" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C35" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D35" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E35" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F35" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G35" t="s">
         <v>8</v>
@@ -2413,20 +2413,20 @@
         <v>6</v>
       </c>
       <c r="B36" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C36" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D36" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E36" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2024</v>
       </c>
       <c r="F36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G36" t="s">
         <v>8</v>
@@ -2452,20 +2452,20 @@
         <v>6</v>
       </c>
       <c r="B37" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C37" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D37" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E37" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F37" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G37" t="s">
         <v>8</v>
@@ -2491,20 +2491,20 @@
         <v>6</v>
       </c>
       <c r="B38" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C38" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D38" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E38" t="str">
         <f>RIGHT(Tabela3[[#This Row],[numero_convenio]],4)</f>
         <v>2022</v>
       </c>
       <c r="F38" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G38" t="s">
         <v>8</v>
@@ -2555,160 +2555,160 @@
         <v>3</v>
       </c>
       <c r="B1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" t="s">
         <v>50</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>51</v>
-      </c>
-      <c r="F1" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" s="2">
-        <v>391415.85</v>
+        <v>101580.66</v>
       </c>
       <c r="D2" s="2">
-        <v>391415.85</v>
+        <v>101580.66</v>
       </c>
       <c r="E2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
       <c r="C3" s="2">
-        <v>391415.85</v>
+        <v>287924.42</v>
       </c>
       <c r="D3" s="2">
-        <v>391415.85</v>
+        <v>287924.42</v>
       </c>
       <c r="E3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
       <c r="C4" s="2">
-        <v>391415.85</v>
+        <v>180717.89</v>
       </c>
       <c r="D4" s="2">
-        <v>391415.85</v>
+        <v>180717.89</v>
       </c>
       <c r="E4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
       <c r="C5" s="2">
-        <v>391415.85</v>
+        <v>308369.88</v>
       </c>
       <c r="D5" s="2">
-        <v>391415.85</v>
+        <v>308369.88</v>
       </c>
       <c r="E5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B6">
         <v>5</v>
       </c>
       <c r="C6" s="2">
-        <v>391415.85</v>
+        <v>220978.86</v>
       </c>
       <c r="D6" s="2">
-        <v>391415.85</v>
+        <v>220978.86</v>
       </c>
       <c r="E6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B7">
         <v>6</v>
       </c>
       <c r="C7" s="2">
-        <v>391415.85</v>
+        <v>578329.38</v>
       </c>
       <c r="D7" s="2">
-        <v>391415.85</v>
+        <v>578329.38</v>
       </c>
       <c r="E7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B8">
         <v>7</v>
       </c>
       <c r="C8" s="2">
-        <v>391415.85</v>
+        <v>555678.85</v>
       </c>
       <c r="D8" s="2">
-        <v>391415.85</v>
+        <v>555678.85</v>
       </c>
       <c r="E8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B9">
         <v>8</v>
       </c>
       <c r="C9" s="2">
-        <v>391415.85</v>
+        <v>631917.94999999995</v>
       </c>
       <c r="D9" s="2">
-        <v>391415.85</v>
+        <v>631917.94999999995</v>
       </c>
       <c r="E9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B10">
         <v>9</v>
@@ -2717,15 +2717,15 @@
         <v>391415.85</v>
       </c>
       <c r="E10" t="s">
+        <v>53</v>
+      </c>
+      <c r="F10" t="s">
         <v>54</v>
-      </c>
-      <c r="F10" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B11">
         <v>10</v>
@@ -2734,12 +2734,12 @@
         <v>159921.1</v>
       </c>
       <c r="E11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B12">
         <v>11</v>
@@ -2748,12 +2748,12 @@
         <v>115504.26</v>
       </c>
       <c r="E12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B13">
         <v>12</v>
@@ -2762,12 +2762,12 @@
         <v>76643.03</v>
       </c>
       <c r="E13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B14">
         <v>1</v>
@@ -2779,131 +2779,131 @@
         <v>1000000</v>
       </c>
       <c r="E14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" s="2">
-        <v>2140606.5299999998</v>
+        <v>2880912.2</v>
       </c>
       <c r="D15" s="2">
-        <v>2140606.5299999998</v>
+        <v>2880912.2</v>
       </c>
       <c r="E15" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B16">
         <v>2</v>
       </c>
       <c r="C16" s="2">
-        <v>2140606.5299999998</v>
+        <v>2880912.2</v>
       </c>
       <c r="D16" s="2">
-        <v>2140606.5299999998</v>
+        <v>2880912.2</v>
       </c>
       <c r="E16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B17">
         <v>3</v>
       </c>
       <c r="C17" s="2">
-        <v>2140606.5299999998</v>
+        <v>2880912.2</v>
       </c>
       <c r="D17" s="2">
-        <v>2140606.5299999998</v>
+        <v>2880912.2</v>
       </c>
       <c r="E17" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B18">
         <v>4</v>
       </c>
       <c r="C18" s="2">
-        <v>2140606.5299999998</v>
+        <v>2880912.2</v>
       </c>
       <c r="D18" s="2">
-        <v>2140606.5299999998</v>
+        <v>2880912.2</v>
       </c>
       <c r="E18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B19">
         <v>5</v>
       </c>
       <c r="C19" s="2">
-        <v>2140606.5299999998</v>
+        <v>2880912.2</v>
       </c>
       <c r="D19" s="2">
-        <v>2140606.5299999998</v>
+        <v>2880912.2</v>
       </c>
       <c r="E19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B20">
         <v>6</v>
       </c>
       <c r="C20" s="2">
-        <v>2140606.5299999998</v>
+        <v>2880912.22</v>
       </c>
       <c r="D20" s="2">
-        <v>2140606.5299999998</v>
+        <v>2880912.22</v>
       </c>
       <c r="E20" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B21">
         <v>7</v>
       </c>
       <c r="C21" s="2">
-        <v>2140606.5299999998</v>
+        <v>2140606.52</v>
       </c>
       <c r="D21" s="2">
-        <v>2140606.5299999998</v>
+        <v>2140606.52</v>
       </c>
       <c r="E21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B22">
         <v>8</v>
@@ -2912,83 +2912,83 @@
         <v>2140606.5299999998</v>
       </c>
       <c r="E22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B23">
         <v>1</v>
       </c>
       <c r="C23" s="2">
-        <v>1198402.5600000001</v>
+        <v>2434904.7799999998</v>
       </c>
       <c r="D23" s="2">
-        <v>1198402.5600000001</v>
+        <v>2434904.7799999998</v>
       </c>
       <c r="E23" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B24">
         <v>2</v>
       </c>
       <c r="C24" s="2">
-        <v>1198402.5600000001</v>
+        <v>2434904.7799999998</v>
       </c>
       <c r="D24" s="2">
-        <v>1198402.5600000001</v>
+        <v>2434904.7799999998</v>
       </c>
       <c r="E24" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B25">
         <v>3</v>
       </c>
       <c r="C25" s="2">
-        <v>1198402.5600000001</v>
+        <v>2434904.7799999998</v>
       </c>
       <c r="D25" s="2">
-        <v>1198402.5600000001</v>
+        <v>2434904.7799999998</v>
       </c>
       <c r="E25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B26">
         <v>4</v>
       </c>
       <c r="C26" s="2">
-        <v>1198402.5600000001</v>
+        <v>2434904.7999999998</v>
       </c>
       <c r="D26" s="2">
-        <v>1198402.5600000001</v>
+        <v>2434904.7999999998</v>
       </c>
       <c r="E26" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B27">
         <v>5</v>
@@ -3000,12 +3000,12 @@
         <v>1198402.5600000001</v>
       </c>
       <c r="E27" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B28">
         <v>6</v>
@@ -3017,12 +3017,12 @@
         <v>1198402.5600000001</v>
       </c>
       <c r="E28" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B29">
         <v>7</v>
@@ -3031,15 +3031,15 @@
         <v>1198402.5600000001</v>
       </c>
       <c r="E29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F29" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B30">
         <v>8</v>
@@ -3048,80 +3048,80 @@
         <v>1198402.5600000001</v>
       </c>
       <c r="E30" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B31">
         <v>1</v>
       </c>
       <c r="C31" s="2">
-        <v>4598922.4400000004</v>
+        <v>4625000</v>
       </c>
       <c r="D31" s="2">
-        <v>4598922.4400000004</v>
+        <v>4625000</v>
       </c>
       <c r="E31" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B32">
         <v>2</v>
       </c>
       <c r="C32" s="2">
-        <v>4598922.4400000004</v>
+        <v>4625000</v>
       </c>
       <c r="D32" s="2">
-        <v>4598922.4400000004</v>
+        <v>4625000</v>
       </c>
       <c r="E32" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B33">
         <v>3</v>
       </c>
       <c r="C33" s="2">
-        <v>4598922.4400000004</v>
+        <v>4625000</v>
       </c>
       <c r="D33" s="2">
-        <v>4598922.4400000004</v>
+        <v>4625000</v>
       </c>
       <c r="E33" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B34">
         <v>4</v>
       </c>
       <c r="C34" s="2">
-        <v>4598922.4400000004</v>
+        <v>4625000</v>
       </c>
       <c r="D34" s="2">
-        <v>4598922.4400000004</v>
+        <v>4625000</v>
       </c>
       <c r="E34" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B35">
         <v>5</v>
@@ -3130,15 +3130,15 @@
         <v>4598922.4400000004</v>
       </c>
       <c r="E35" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F35" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B36">
         <v>1</v>
@@ -3150,12 +3150,12 @@
         <v>464005.33</v>
       </c>
       <c r="E36" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B37">
         <v>2</v>
@@ -3167,12 +3167,12 @@
         <v>464005.33</v>
       </c>
       <c r="E37" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B38">
         <v>3</v>
@@ -3181,15 +3181,15 @@
         <v>464005.33</v>
       </c>
       <c r="E38" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F38" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B39">
         <v>1</v>
@@ -3201,12 +3201,12 @@
         <v>250000</v>
       </c>
       <c r="E39" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B40">
         <v>2</v>
@@ -3218,12 +3218,12 @@
         <v>250000</v>
       </c>
       <c r="E40" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B41">
         <v>1</v>
@@ -3235,12 +3235,12 @@
         <v>250000</v>
       </c>
       <c r="E41" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B42">
         <v>2</v>
@@ -3252,12 +3252,12 @@
         <v>250000</v>
       </c>
       <c r="E42" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B43">
         <v>1</v>
@@ -3269,12 +3269,12 @@
         <v>1473325.6</v>
       </c>
       <c r="E43" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B44">
         <v>2</v>
@@ -3286,12 +3286,12 @@
         <v>1473325.6</v>
       </c>
       <c r="E44" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B45">
         <v>3</v>
@@ -3303,12 +3303,12 @@
         <v>1473325.6</v>
       </c>
       <c r="E45" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B46">
         <v>4</v>
@@ -3320,12 +3320,12 @@
         <v>1473325.6</v>
       </c>
       <c r="E46" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B47">
         <v>5</v>
@@ -3337,80 +3337,80 @@
         <v>1473325.6</v>
       </c>
       <c r="E47" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B48">
         <v>1</v>
       </c>
       <c r="C48" s="2">
-        <v>941635.57</v>
+        <v>1561412.1</v>
       </c>
       <c r="D48" s="2">
-        <v>941635.57</v>
+        <v>1561412.1</v>
       </c>
       <c r="E48" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B49">
         <v>2</v>
       </c>
       <c r="C49" s="2">
-        <v>941635.57</v>
+        <v>1561412.1</v>
       </c>
       <c r="D49" s="2">
-        <v>941635.57</v>
+        <v>1561412.1</v>
       </c>
       <c r="E49" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B50">
         <v>3</v>
       </c>
       <c r="C50" s="2">
-        <v>941635.57</v>
+        <v>1561412.1</v>
       </c>
       <c r="D50" s="2">
-        <v>941635.57</v>
+        <v>1561412.1</v>
       </c>
       <c r="E50" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B51">
         <v>4</v>
       </c>
       <c r="C51" s="2">
-        <v>941635.57</v>
+        <v>1561412.11</v>
       </c>
       <c r="D51" s="2">
-        <v>941635.57</v>
+        <v>1561412.11</v>
       </c>
       <c r="E51" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B52">
         <v>5</v>
@@ -3419,12 +3419,12 @@
         <v>941635.57</v>
       </c>
       <c r="E52" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B53">
         <v>6</v>
@@ -3433,15 +3433,15 @@
         <v>941635.57</v>
       </c>
       <c r="E53" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F53" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B54">
         <v>1</v>
@@ -3453,12 +3453,12 @@
         <v>2993434.29</v>
       </c>
       <c r="E54" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B55">
         <v>2</v>
@@ -3470,12 +3470,12 @@
         <v>2993434.29</v>
       </c>
       <c r="E55" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B56">
         <v>3</v>
@@ -3487,12 +3487,12 @@
         <v>2993434.29</v>
       </c>
       <c r="E56" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B57">
         <v>4</v>
@@ -3504,63 +3504,63 @@
         <v>2993434.29</v>
       </c>
       <c r="E57" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B58">
         <v>1</v>
       </c>
       <c r="C58" s="2">
-        <v>2209930.54</v>
+        <v>2209930.5499999998</v>
       </c>
       <c r="D58" s="2">
-        <v>2209930.54</v>
+        <v>2209930.5499999998</v>
       </c>
       <c r="E58" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B59">
         <v>2</v>
       </c>
       <c r="C59" s="2">
-        <v>2209930.54</v>
+        <v>3314895.81</v>
       </c>
       <c r="D59" s="2">
-        <v>2209930.54</v>
+        <v>3314895.81</v>
       </c>
       <c r="E59" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B60">
         <v>3</v>
       </c>
       <c r="C60" s="2">
-        <v>2209930.54</v>
+        <v>3314895.81</v>
       </c>
       <c r="D60" s="2">
-        <v>2209930.54</v>
+        <v>3314895.81</v>
       </c>
       <c r="E60" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B61">
         <v>4</v>
@@ -3569,49 +3569,49 @@
         <v>2209930.54</v>
       </c>
       <c r="E61" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F61" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B62">
         <v>1</v>
       </c>
       <c r="C62" s="2">
-        <v>134390.48000000001</v>
+        <v>335976.19</v>
       </c>
       <c r="D62" s="2">
-        <v>134390.48000000001</v>
+        <v>335976.19</v>
       </c>
       <c r="E62" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B63">
         <v>2</v>
       </c>
       <c r="C63" s="2">
-        <v>134390.48000000001</v>
+        <v>201585.71</v>
       </c>
       <c r="D63" s="2">
-        <v>134390.48000000001</v>
+        <v>201585.71</v>
       </c>
       <c r="E63" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B64">
         <v>3</v>
@@ -3620,15 +3620,15 @@
         <v>134390.48000000001</v>
       </c>
       <c r="E64" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F64" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B65">
         <v>1</v>
@@ -3640,12 +3640,12 @@
         <v>600000</v>
       </c>
       <c r="E65" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B66">
         <v>2</v>
@@ -3657,12 +3657,12 @@
         <v>600000</v>
       </c>
       <c r="E66" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B67">
         <v>3</v>
@@ -3674,63 +3674,63 @@
         <v>600000</v>
       </c>
       <c r="E67" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B68">
         <v>1</v>
       </c>
       <c r="C68" s="2">
-        <v>855664.06</v>
+        <v>1634225.9</v>
       </c>
       <c r="D68" s="2">
-        <v>855664.06</v>
+        <v>1634225.9</v>
       </c>
       <c r="E68" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B69">
         <v>2</v>
       </c>
       <c r="C69" s="2">
-        <v>855664.06</v>
+        <v>1656406.24</v>
       </c>
       <c r="D69" s="2">
-        <v>855664.06</v>
+        <v>1656406.24</v>
       </c>
       <c r="E69" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B70">
         <v>3</v>
       </c>
       <c r="C70" s="2">
-        <v>855664.06</v>
+        <v>1844090.34</v>
       </c>
       <c r="D70" s="2">
-        <v>855664.06</v>
+        <v>1844090.34</v>
       </c>
       <c r="E70" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B71">
         <v>4</v>
@@ -3742,12 +3742,12 @@
         <v>855664.06</v>
       </c>
       <c r="E71" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B72">
         <v>5</v>
@@ -3756,15 +3756,15 @@
         <v>855664.06</v>
       </c>
       <c r="E72" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F72" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B73">
         <v>1</v>
@@ -3776,63 +3776,63 @@
         <v>200860.2</v>
       </c>
       <c r="E73" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B74">
         <v>1</v>
       </c>
       <c r="C74" s="2">
-        <v>410305.24</v>
+        <v>157680.35999999999</v>
       </c>
       <c r="D74" s="2">
-        <v>410305.24</v>
+        <v>157680.35999999999</v>
       </c>
       <c r="E74" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B75">
         <v>2</v>
       </c>
       <c r="C75" s="2">
-        <v>410305.24</v>
+        <v>271298.92</v>
       </c>
       <c r="D75" s="2">
-        <v>410305.24</v>
+        <v>271298.92</v>
       </c>
       <c r="E75" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B76">
         <v>3</v>
       </c>
       <c r="C76" s="2">
-        <v>410305.24</v>
+        <v>164789.91</v>
       </c>
       <c r="D76" s="2">
-        <v>410305.24</v>
+        <v>164789.91</v>
       </c>
       <c r="E76" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B77">
         <v>4</v>
@@ -3841,15 +3841,15 @@
         <v>410305.24</v>
       </c>
       <c r="E77" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F77" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B78">
         <v>1</v>
@@ -3861,12 +3861,12 @@
         <v>990000</v>
       </c>
       <c r="E78" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B79">
         <v>2</v>
@@ -3878,12 +3878,12 @@
         <v>990000</v>
       </c>
       <c r="E79" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B80">
         <v>3</v>
@@ -3895,12 +3895,12 @@
         <v>990000</v>
       </c>
       <c r="E80" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B81">
         <v>4</v>
@@ -3912,12 +3912,12 @@
         <v>990000</v>
       </c>
       <c r="E81" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B82">
         <v>1</v>
@@ -3929,12 +3929,12 @@
         <v>1880137.81</v>
       </c>
       <c r="E82" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B83">
         <v>2</v>
@@ -3946,12 +3946,12 @@
         <v>1880137.81</v>
       </c>
       <c r="E83" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B84">
         <v>3</v>
@@ -3963,12 +3963,12 @@
         <v>1880137.81</v>
       </c>
       <c r="E84" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B85">
         <v>4</v>
@@ -3980,12 +3980,12 @@
         <v>1880137.81</v>
       </c>
       <c r="E85" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B86">
         <v>5</v>
@@ -3997,12 +3997,12 @@
         <v>1880137.81</v>
       </c>
       <c r="E86" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B87">
         <v>6</v>
@@ -4011,66 +4011,66 @@
         <v>1880137.81</v>
       </c>
       <c r="E87" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F87" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B88">
         <v>1</v>
       </c>
       <c r="C88" s="2">
-        <v>328423.7</v>
+        <v>205161.07</v>
       </c>
       <c r="D88" s="2">
-        <v>328423.7</v>
+        <v>205161.07</v>
       </c>
       <c r="E88" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B89">
         <v>2</v>
       </c>
       <c r="C89" s="2">
-        <v>328423.7</v>
+        <v>341935.12</v>
       </c>
       <c r="D89" s="2">
-        <v>328423.7</v>
+        <v>341935.12</v>
       </c>
       <c r="E89" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B90">
         <v>3</v>
       </c>
       <c r="C90" s="2">
-        <v>328423.7</v>
+        <v>136774.04</v>
       </c>
       <c r="D90" s="2">
-        <v>328423.7</v>
+        <v>136774.04</v>
       </c>
       <c r="E90" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B91">
         <v>4</v>
@@ -4079,100 +4079,100 @@
         <v>328423.7</v>
       </c>
       <c r="E91" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F91" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B92">
         <v>1</v>
       </c>
       <c r="C92" s="2">
-        <v>3988000.04</v>
+        <v>2500000</v>
       </c>
       <c r="D92" s="2">
-        <v>3988000.04</v>
+        <v>2500000</v>
       </c>
       <c r="E92" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B93">
         <v>2</v>
       </c>
       <c r="C93" s="2">
-        <v>3988000.04</v>
+        <v>3988000.01</v>
       </c>
       <c r="D93" s="2">
-        <v>3988000.04</v>
+        <v>3988000.01</v>
       </c>
       <c r="E93" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B94">
         <v>3</v>
       </c>
       <c r="C94" s="2">
-        <v>3988000.04</v>
+        <v>3988000.01</v>
       </c>
       <c r="D94" s="2">
-        <v>3988000.04</v>
+        <v>3988000.01</v>
       </c>
       <c r="E94" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B95">
         <v>4</v>
       </c>
       <c r="C95" s="2">
-        <v>3988000.04</v>
+        <v>3988000.01</v>
       </c>
       <c r="D95" s="2">
-        <v>3988000.04</v>
+        <v>3988000.01</v>
       </c>
       <c r="E95" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B96">
         <v>5</v>
       </c>
       <c r="C96" s="2">
-        <v>3988000.04</v>
+        <v>3988000.01</v>
       </c>
       <c r="D96" s="2">
-        <v>3988000.04</v>
+        <v>3988000.01</v>
       </c>
       <c r="E96" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B97">
         <v>6</v>
@@ -4181,15 +4181,15 @@
         <v>3988000.04</v>
       </c>
       <c r="E97" t="s">
+        <v>61</v>
+      </c>
+      <c r="F97" t="s">
         <v>62</v>
-      </c>
-      <c r="F97" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B98">
         <v>7</v>
@@ -4198,29 +4198,29 @@
         <v>5385600.0199999996</v>
       </c>
       <c r="E98" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B99">
         <v>1</v>
       </c>
       <c r="C99" s="2">
-        <v>144000</v>
+        <v>465600</v>
       </c>
       <c r="D99" s="2">
-        <v>144000</v>
+        <v>465600</v>
       </c>
       <c r="E99" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B100">
         <v>2</v>
@@ -4229,15 +4229,15 @@
         <v>144000</v>
       </c>
       <c r="E100" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F100" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B101">
         <v>1</v>
@@ -4249,12 +4249,12 @@
         <v>2965467.43</v>
       </c>
       <c r="E101" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B102">
         <v>2</v>
@@ -4266,12 +4266,12 @@
         <v>2965467.43</v>
       </c>
       <c r="E102" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B103">
         <v>3</v>
@@ -4283,12 +4283,12 @@
         <v>2965467.43</v>
       </c>
       <c r="E103" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B104">
         <v>4</v>
@@ -4300,12 +4300,12 @@
         <v>2965467.43</v>
       </c>
       <c r="E104" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B105">
         <v>5</v>
@@ -4314,12 +4314,12 @@
         <v>2965467.43</v>
       </c>
       <c r="E105" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B106">
         <v>6</v>
@@ -4328,117 +4328,117 @@
         <v>2965467.43</v>
       </c>
       <c r="E106" t="s">
+        <v>61</v>
+      </c>
+      <c r="F106" t="s">
         <v>62</v>
-      </c>
-      <c r="F106" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B107">
         <v>1</v>
       </c>
       <c r="C107" s="2">
-        <v>521425.52</v>
+        <v>170025.32</v>
       </c>
       <c r="D107" s="2">
-        <v>521425.52</v>
+        <v>170025.32</v>
       </c>
       <c r="E107" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B108">
         <v>2</v>
       </c>
       <c r="C108" s="2">
-        <v>521425.52</v>
+        <v>374574.7</v>
       </c>
       <c r="D108" s="2">
-        <v>521425.52</v>
+        <v>374574.7</v>
       </c>
       <c r="E108" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B109">
         <v>3</v>
       </c>
       <c r="C109" s="2">
-        <v>521425.52</v>
+        <v>388435.68</v>
       </c>
       <c r="D109" s="2">
-        <v>521425.52</v>
+        <v>388435.68</v>
       </c>
       <c r="E109" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B110">
         <v>4</v>
       </c>
       <c r="C110" s="2">
-        <v>521425.52</v>
+        <v>456886.58</v>
       </c>
       <c r="D110" s="2">
-        <v>521425.52</v>
+        <v>456886.58</v>
       </c>
       <c r="E110" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B111">
         <v>5</v>
       </c>
       <c r="C111" s="2">
-        <v>521425.52</v>
+        <v>700834.08</v>
       </c>
       <c r="D111" s="2">
-        <v>521425.52</v>
+        <v>700834.08</v>
       </c>
       <c r="E111" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B112">
         <v>6</v>
       </c>
       <c r="C112" s="2">
-        <v>521425.52</v>
+        <v>780863.16</v>
       </c>
       <c r="D112" s="2">
-        <v>521425.52</v>
+        <v>780863.16</v>
       </c>
       <c r="E112" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B113">
         <v>7</v>
@@ -4447,94 +4447,94 @@
         <v>521425.52</v>
       </c>
       <c r="E113" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B114">
         <v>8</v>
       </c>
       <c r="C114" s="2">
-        <v>521425.52</v>
+        <v>521425.53</v>
       </c>
       <c r="E114" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F114" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B115">
         <v>1</v>
       </c>
       <c r="C115" s="2">
-        <v>480000</v>
+        <v>600000</v>
       </c>
       <c r="D115" s="2">
-        <v>480000</v>
+        <v>600000</v>
       </c>
       <c r="E115" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B116">
         <v>2</v>
       </c>
       <c r="C116" s="2">
-        <v>480000</v>
+        <v>600000</v>
       </c>
       <c r="D116" s="2">
-        <v>480000</v>
+        <v>600000</v>
       </c>
       <c r="E116" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B117">
         <v>3</v>
       </c>
       <c r="C117" s="2">
-        <v>480000</v>
+        <v>600000</v>
       </c>
       <c r="D117" s="2">
-        <v>480000</v>
+        <v>600000</v>
       </c>
       <c r="E117" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B118">
         <v>4</v>
       </c>
       <c r="C118" s="2">
-        <v>480000</v>
+        <v>600000</v>
       </c>
       <c r="E118" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B119">
         <v>5</v>
@@ -4543,15 +4543,15 @@
         <v>480000</v>
       </c>
       <c r="E119" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F119" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B120">
         <v>1</v>
@@ -4563,12 +4563,12 @@
         <v>3241338.27</v>
       </c>
       <c r="E120" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B121">
         <v>2</v>
@@ -4580,12 +4580,12 @@
         <v>3241338.27</v>
       </c>
       <c r="E121" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B122">
         <v>3</v>
@@ -4597,12 +4597,12 @@
         <v>3241338.27</v>
       </c>
       <c r="E122" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B123">
         <v>1</v>
@@ -4614,12 +4614,12 @@
         <v>238943.16</v>
       </c>
       <c r="E123" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B124">
         <v>1</v>
@@ -4631,12 +4631,12 @@
         <v>1615786.09</v>
       </c>
       <c r="E124" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B125">
         <v>1</v>
@@ -4648,12 +4648,12 @@
         <v>992349.34</v>
       </c>
       <c r="E125" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B126">
         <v>1</v>
@@ -4665,12 +4665,12 @@
         <v>131846.39999999999</v>
       </c>
       <c r="E126" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B127">
         <v>1</v>
@@ -4682,12 +4682,12 @@
         <v>607929.73</v>
       </c>
       <c r="E127" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B128">
         <v>1</v>
@@ -4699,29 +4699,29 @@
         <v>990812.45</v>
       </c>
       <c r="E128" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B129">
         <v>1</v>
       </c>
       <c r="C129" s="2">
-        <v>4094327.45</v>
+        <v>3794475.99</v>
       </c>
       <c r="D129" s="2">
-        <v>4094327.45</v>
+        <v>3794475.99</v>
       </c>
       <c r="E129" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B130">
         <v>2</v>
@@ -4730,15 +4730,15 @@
         <v>4094327.45</v>
       </c>
       <c r="E130" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F130" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B131">
         <v>3</v>
@@ -4747,12 +4747,12 @@
         <v>3306736.66</v>
       </c>
       <c r="E131" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B132">
         <v>4</v>
@@ -4761,12 +4761,12 @@
         <v>2186682.88</v>
       </c>
       <c r="E132" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B133">
         <v>1</v>
@@ -4778,12 +4778,12 @@
         <v>286440</v>
       </c>
       <c r="E133" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B134">
         <v>1</v>
@@ -4795,12 +4795,12 @@
         <v>3000000</v>
       </c>
       <c r="E134" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B135">
         <v>2</v>
@@ -4812,12 +4812,12 @@
         <v>3000000</v>
       </c>
       <c r="E135" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B136">
         <v>3</v>
@@ -4829,12 +4829,12 @@
         <v>3000000</v>
       </c>
       <c r="E136" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B137">
         <v>4</v>
@@ -4846,12 +4846,12 @@
         <v>3000000</v>
       </c>
       <c r="E137" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B138">
         <v>5</v>
@@ -4863,12 +4863,12 @@
         <v>3000000</v>
       </c>
       <c r="E138" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B139">
         <v>6</v>
@@ -4880,12 +4880,12 @@
         <v>3000000</v>
       </c>
       <c r="E139" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B140">
         <v>7</v>
@@ -4894,15 +4894,15 @@
         <v>3000000</v>
       </c>
       <c r="E140" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F140" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B141">
         <v>8</v>
@@ -4911,12 +4911,12 @@
         <v>3000000</v>
       </c>
       <c r="E141" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B142">
         <v>9</v>
@@ -4925,12 +4925,12 @@
         <v>3000000</v>
       </c>
       <c r="E142" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B143">
         <v>10</v>
@@ -4939,12 +4939,12 @@
         <v>3000000</v>
       </c>
       <c r="E143" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B144">
         <v>1</v>
@@ -4953,15 +4953,15 @@
         <v>100000</v>
       </c>
       <c r="E144" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F144" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B145">
         <v>1</v>
@@ -4970,10 +4970,10 @@
         <v>200000</v>
       </c>
       <c r="E145" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F145" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -4998,351 +4998,351 @@
         <v>3</v>
       </c>
       <c r="B1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B16" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B18" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B20" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B21" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B22" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B24" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B25" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B26" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B27" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B28" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B29" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B30" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B31" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B32" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B33" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B34" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B35" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B36" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B37" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B38" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B39" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B40" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B41" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B42" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B43" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B44" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>

</xml_diff>